<commit_message>
Implementar un módulo de gestión financiera con funciones de seguimiento de transacciones, presupuesto y objetivos.
</commit_message>
<xml_diff>
--- a/Docs/Cronograma/Cronograma FinanzaViva.xlsx
+++ b/Docs/Cronograma/Cronograma FinanzaViva.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felipe\Desktop\FinanzaViva\Docs\Cronograma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64739A48-8EE8-4230-B0F8-767AB4AA14F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBB2C63-B150-4493-8B75-B9E90CD28C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -111,9 +111,6 @@
     <t>Módulo Quizzes (preguntas, recompensas)</t>
   </si>
   <si>
-    <t>Módulo Simulador financiero (turnos, multijugador)</t>
-  </si>
-  <si>
     <t>Módulo Dashboard (resumen, estadísticas)</t>
   </si>
   <si>
@@ -149,20 +146,11 @@
     <t>Integración backend-frontend por módulo</t>
   </si>
   <si>
-    <t>Pruebas unitarias backend (Jest)</t>
-  </si>
-  <si>
-    <t>Pruebas E2E y flujos completos</t>
-  </si>
-  <si>
     <t>Corrección de bugs y refinamiento</t>
   </si>
   <si>
     <t>6. Documentación
 &amp; Despliegue</t>
-  </si>
-  <si>
-    <t>Documentación técnica (API, arquitectura)</t>
   </si>
   <si>
     <t>Manual de usuario y guía de instalación</t>
@@ -226,6 +214,18 @@
   </si>
   <si>
     <t>Felipe Molina</t>
+  </si>
+  <si>
+    <t>Módulo Simulador financiero (turnos, multijugador local)</t>
+  </si>
+  <si>
+    <t>Pruebas de flujos completos</t>
+  </si>
+  <si>
+    <t>Pruebas unitarias backend</t>
+  </si>
+  <si>
+    <t>Documentación técnica</t>
   </si>
 </sst>
 </file>
@@ -542,19 +542,81 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -563,68 +625,6 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -948,75 +948,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="16"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
+      <c r="P1" s="41"/>
+      <c r="Q1" s="41"/>
+      <c r="R1" s="41"/>
+      <c r="S1" s="41"/>
+      <c r="T1" s="41"/>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="29" t="s">
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="18" t="s">
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="18" t="s">
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="20"/>
-      <c r="T2" s="17" t="s">
+      <c r="Q2" s="28"/>
+      <c r="R2" s="28"/>
+      <c r="S2" s="42"/>
+      <c r="T2" s="39" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="34"/>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
+      <c r="A3" s="38"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
       <c r="D3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="40" t="s">
+      <c r="E3" s="20" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -1031,7 +1031,7 @@
       <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="40" t="s">
+      <c r="J3" s="20" t="s">
         <v>11</v>
       </c>
       <c r="K3" s="13" t="s">
@@ -1061,21 +1061,21 @@
       <c r="S3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="T3" s="41" t="s">
+      <c r="T3" s="21" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
-        <v>49</v>
+      <c r="A4" s="43" t="s">
+        <v>45</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="42"/>
+      <c r="C4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="22"/>
       <c r="E4" s="12"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -1094,14 +1094,14 @@
       <c r="T4" s="6"/>
     </row>
     <row r="5" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="21"/>
+      <c r="A5" s="43"/>
       <c r="B5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" s="42"/>
+      <c r="C5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="22"/>
       <c r="E5" s="12"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -1120,14 +1120,14 @@
       <c r="T5" s="6"/>
     </row>
     <row r="6" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21"/>
+      <c r="A6" s="43"/>
       <c r="B6" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D6" s="42"/>
+        <v>42</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="22"/>
       <c r="E6" s="12"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -1146,14 +1146,14 @@
       <c r="T6" s="6"/>
     </row>
     <row r="7" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="21"/>
+      <c r="A7" s="43"/>
       <c r="B7" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="42"/>
+        <v>43</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="22"/>
       <c r="E7" s="6"/>
       <c r="F7" s="12"/>
       <c r="G7" s="6"/>
@@ -1172,14 +1172,14 @@
       <c r="T7" s="6"/>
     </row>
     <row r="8" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="21"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="42"/>
+      <c r="C8" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="22"/>
       <c r="E8" s="6"/>
       <c r="F8" s="12"/>
       <c r="G8" s="6"/>
@@ -1198,14 +1198,14 @@
       <c r="T8" s="6"/>
     </row>
     <row r="9" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="21"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" s="42"/>
+      <c r="C9" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="22"/>
       <c r="E9" s="6"/>
       <c r="F9" s="12"/>
       <c r="G9" s="6"/>
@@ -1224,14 +1224,14 @@
       <c r="T9" s="6"/>
     </row>
     <row r="10" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="21"/>
+      <c r="A10" s="43"/>
       <c r="B10" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="D10" s="42"/>
+        <v>44</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="22"/>
       <c r="E10" s="6"/>
       <c r="F10" s="12"/>
       <c r="G10" s="6"/>
@@ -1250,21 +1250,21 @@
       <c r="T10" s="6"/>
     </row>
     <row r="11" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>51</v>
+      <c r="A11" s="24" t="s">
+        <v>47</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="38" t="s">
-        <v>59</v>
+        <v>50</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>55</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
-      <c r="J11" s="42"/>
+      <c r="J11" s="22"/>
       <c r="K11" s="6"/>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
@@ -1277,12 +1277,12 @@
       <c r="T11" s="6"/>
     </row>
     <row r="12" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
+      <c r="A12" s="24"/>
       <c r="B12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="17" t="s">
         <v>55</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>59</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="6"/>
@@ -1290,7 +1290,7 @@
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
-      <c r="J12" s="42"/>
+      <c r="J12" s="22"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
       <c r="M12" s="6"/>
@@ -1303,14 +1303,14 @@
       <c r="T12" s="6"/>
     </row>
     <row r="13" spans="1:20" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="22"/>
+      <c r="A13" s="24"/>
       <c r="B13" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="D13" s="42"/>
+        <v>52</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="22"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
@@ -1329,16 +1329,16 @@
       <c r="T13" s="6"/>
     </row>
     <row r="14" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="35" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="42"/>
+      <c r="C14" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="22"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
       <c r="G14" s="12"/>
@@ -1357,14 +1357,14 @@
       <c r="T14" s="6"/>
     </row>
     <row r="15" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="32"/>
+      <c r="A15" s="36"/>
       <c r="B15" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D15" s="42"/>
+      <c r="C15" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="22"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
       <c r="G15" s="12"/>
@@ -1383,14 +1383,14 @@
       <c r="T15" s="6"/>
     </row>
     <row r="16" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="32"/>
+      <c r="A16" s="36"/>
       <c r="B16" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="42"/>
+      <c r="C16" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="22"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
       <c r="G16" s="12"/>
@@ -1409,14 +1409,14 @@
       <c r="T16" s="6"/>
     </row>
     <row r="17" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="32"/>
+      <c r="A17" s="36"/>
       <c r="B17" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D17" s="42"/>
+      <c r="C17" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="22"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
@@ -1435,14 +1435,14 @@
       <c r="T17" s="6"/>
     </row>
     <row r="18" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="32"/>
+      <c r="A18" s="36"/>
       <c r="B18" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="42"/>
+      <c r="C18" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="22"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
@@ -1461,14 +1461,14 @@
       <c r="T18" s="6"/>
     </row>
     <row r="19" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="32"/>
+      <c r="A19" s="36"/>
       <c r="B19" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D19" s="42"/>
+      <c r="C19" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="22"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
@@ -1487,19 +1487,18 @@
       <c r="T19" s="6"/>
     </row>
     <row r="20" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="32"/>
+      <c r="A20" s="36"/>
       <c r="B20" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="42"/>
+        <v>57</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="22"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="12"/>
+      <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
       <c r="L20" s="6"/>
@@ -1513,14 +1512,14 @@
       <c r="T20" s="6"/>
     </row>
     <row r="21" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="32"/>
+      <c r="A21" s="36"/>
       <c r="B21" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="42"/>
+        <v>24</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="22"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
@@ -1539,16 +1538,16 @@
       <c r="T21" s="6"/>
     </row>
     <row r="22" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="27" t="s">
+      <c r="A22" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C22" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="42"/>
+      <c r="C22" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="22"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
@@ -1567,14 +1566,14 @@
       <c r="T22" s="6"/>
     </row>
     <row r="23" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="28"/>
+      <c r="A23" s="32"/>
       <c r="B23" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D23" s="42"/>
+        <v>27</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" s="22"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
@@ -1593,14 +1592,14 @@
       <c r="T23" s="6"/>
     </row>
     <row r="24" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="28"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="D24" s="42"/>
+        <v>28</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="22"/>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
@@ -1619,14 +1618,14 @@
       <c r="T24" s="6"/>
     </row>
     <row r="25" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="28"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C25" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25" s="42"/>
+        <v>29</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" s="22"/>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
@@ -1634,7 +1633,7 @@
       <c r="I25" s="6"/>
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
-      <c r="L25" s="42"/>
+      <c r="L25" s="22"/>
       <c r="M25" s="6"/>
       <c r="N25" s="6"/>
       <c r="O25" s="6"/>
@@ -1645,14 +1644,14 @@
       <c r="T25" s="6"/>
     </row>
     <row r="26" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="28"/>
+      <c r="A26" s="32"/>
       <c r="B26" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="D26" s="42"/>
+        <v>30</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="22"/>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
@@ -1671,14 +1670,14 @@
       <c r="T26" s="6"/>
     </row>
     <row r="27" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="28"/>
+      <c r="A27" s="32"/>
       <c r="B27" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="D27" s="42"/>
+        <v>31</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" s="22"/>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
@@ -1697,14 +1696,14 @@
       <c r="T27" s="6"/>
     </row>
     <row r="28" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
+      <c r="A28" s="32"/>
       <c r="B28" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D28" s="42"/>
+        <v>32</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" s="22"/>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
       <c r="G28" s="6"/>
@@ -1723,16 +1722,16 @@
       <c r="T28" s="6"/>
     </row>
     <row r="29" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C29" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D29" s="42"/>
+      <c r="C29" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="22"/>
       <c r="E29" s="6"/>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
@@ -1751,14 +1750,14 @@
       <c r="T29" s="6"/>
     </row>
     <row r="30" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="26"/>
+      <c r="A30" s="30"/>
       <c r="B30" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="37" t="s">
-        <v>60</v>
-      </c>
-      <c r="D30" s="42"/>
+        <v>59</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" s="22"/>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
@@ -1777,14 +1776,14 @@
       <c r="T30" s="6"/>
     </row>
     <row r="31" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="26"/>
+      <c r="A31" s="30"/>
       <c r="B31" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D31" s="42"/>
+        <v>58</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="22"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
@@ -1803,14 +1802,14 @@
       <c r="T31" s="6"/>
     </row>
     <row r="32" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="26"/>
+      <c r="A32" s="30"/>
       <c r="B32" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="42"/>
+        <v>35</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D32" s="22"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
@@ -1829,16 +1828,16 @@
       <c r="T32" s="6"/>
     </row>
     <row r="33" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="23" t="s">
-        <v>39</v>
+      <c r="A33" s="25" t="s">
+        <v>36</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C33" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="D33" s="42"/>
+        <v>60</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D33" s="22"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
@@ -1857,14 +1856,14 @@
       <c r="T33" s="6"/>
     </row>
     <row r="34" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="24"/>
+      <c r="A34" s="26"/>
       <c r="B34" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C34" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="D34" s="42"/>
+        <v>37</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D34" s="22"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
@@ -1883,14 +1882,14 @@
       <c r="T34" s="6"/>
     </row>
     <row r="35" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="24"/>
+      <c r="A35" s="26"/>
       <c r="B35" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C35" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="D35" s="42"/>
+        <v>38</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" s="22"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
@@ -1909,22 +1908,22 @@
       <c r="T35" s="6"/>
     </row>
     <row r="36" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="22" t="s">
-        <v>52</v>
+      <c r="A36" s="24" t="s">
+        <v>48</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C36" s="37" t="s">
-        <v>59</v>
+        <v>50</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>55</v>
       </c>
       <c r="D36" s="12"/>
-      <c r="E36" s="42"/>
+      <c r="E36" s="22"/>
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
       <c r="I36" s="6"/>
-      <c r="J36" s="42"/>
+      <c r="J36" s="22"/>
       <c r="K36" s="6"/>
       <c r="L36" s="6"/>
       <c r="M36" s="6"/>
@@ -1937,14 +1936,14 @@
       <c r="T36" s="6"/>
     </row>
     <row r="37" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="22"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C37" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="D37" s="42"/>
+        <v>54</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D37" s="22"/>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
@@ -1963,14 +1962,14 @@
       <c r="T37" s="6"/>
     </row>
     <row r="38" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="22"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C38" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="D38" s="42"/>
+        <v>53</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D38" s="22"/>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
@@ -1990,15 +1989,15 @@
     </row>
     <row r="39" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="D39" s="42"/>
+        <v>39</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D39" s="22"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
@@ -2018,10 +2017,10 @@
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B42" s="43" t="s">
-        <v>45</v>
+        <v>40</v>
+      </c>
+      <c r="B42" s="23" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="69" spans="3:4" x14ac:dyDescent="0.3">
@@ -2042,6 +2041,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="T2"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="A4:A10"/>
+    <mergeCell ref="A11:A13"/>
     <mergeCell ref="A36:A38"/>
     <mergeCell ref="A33:A35"/>
     <mergeCell ref="L2:O2"/>
@@ -2053,11 +2057,6 @@
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="D2:G2"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="T2"/>
-    <mergeCell ref="P2:S2"/>
-    <mergeCell ref="A4:A10"/>
-    <mergeCell ref="A11:A13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="50" orientation="portrait" r:id="rId1"/>

</xml_diff>